<commit_message>
Add a Markdown table export of the register
- scripts/export-legal-register-xlsx.py also writes docs/legal-acts/export-md/*.md,
  one Markdown table per register document with the same columns as the workbooks
- a provision text repeated from the previous row (a whole annex shown for
  several points) is written once and marked instead of duplicated
- classify the row type per act kind: Article, Section, Annex point, Point, Requirement
</commit_message>
<xml_diff>
--- a/docs/legal-acts/export/ETSI TS 119 101.xlsx
+++ b/docs/legal-acts/export/ETSI TS 119 101.xlsx
@@ -473,7 +473,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 18:24</t>
+          <t>2026-10-21 18:31</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr"/>
@@ -870,7 +870,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr"/>
@@ -959,7 +959,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr"/>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr"/>
@@ -1695,7 +1695,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr"/>
@@ -2342,7 +2342,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr"/>
@@ -2431,7 +2431,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr"/>
@@ -2520,7 +2520,7 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr"/>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr"/>
@@ -2698,7 +2698,7 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr"/>
@@ -2787,7 +2787,7 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr"/>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr"/>
@@ -2965,7 +2965,7 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr"/>
@@ -3054,7 +3054,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr"/>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr"/>
@@ -3232,7 +3232,7 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr"/>
@@ -3321,7 +3321,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr"/>
@@ -3410,7 +3410,7 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr"/>
@@ -3499,7 +3499,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr"/>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr"/>
@@ -3677,7 +3677,7 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr"/>
@@ -3766,7 +3766,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr"/>
@@ -3855,7 +3855,7 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr"/>
@@ -3944,7 +3944,7 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr"/>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr"/>
@@ -4122,7 +4122,7 @@
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr"/>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr"/>
@@ -4300,7 +4300,7 @@
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr"/>
@@ -4389,7 +4389,7 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr"/>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr"/>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr"/>
@@ -4656,7 +4656,7 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr"/>
@@ -4745,7 +4745,7 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr"/>
@@ -4834,7 +4834,7 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr"/>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr"/>
@@ -5012,7 +5012,7 @@
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr"/>
@@ -5101,7 +5101,7 @@
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr"/>
@@ -5190,7 +5190,7 @@
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr"/>
@@ -5279,7 +5279,7 @@
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr"/>
@@ -5368,7 +5368,7 @@
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr"/>
@@ -5457,7 +5457,7 @@
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr"/>
@@ -5546,7 +5546,7 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr"/>
@@ -5635,7 +5635,7 @@
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr"/>
@@ -5724,7 +5724,7 @@
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr"/>
@@ -5813,7 +5813,7 @@
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr"/>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr"/>
@@ -5991,7 +5991,7 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr"/>
@@ -6080,7 +6080,7 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr"/>
@@ -6169,7 +6169,7 @@
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr"/>
@@ -6258,7 +6258,7 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr"/>
@@ -6347,7 +6347,7 @@
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr"/>
@@ -6436,7 +6436,7 @@
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr"/>
@@ -6525,7 +6525,7 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr"/>
@@ -6614,7 +6614,7 @@
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr"/>
@@ -6703,7 +6703,7 @@
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr"/>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr"/>
@@ -6881,7 +6881,7 @@
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr"/>
@@ -6970,7 +6970,7 @@
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr"/>
@@ -7059,7 +7059,7 @@
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr"/>
@@ -7148,7 +7148,7 @@
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr"/>
@@ -7237,7 +7237,7 @@
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr"/>
@@ -7326,7 +7326,7 @@
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr"/>
@@ -7415,7 +7415,7 @@
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr"/>
@@ -7504,7 +7504,7 @@
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr"/>
@@ -7593,7 +7593,7 @@
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr"/>
@@ -7682,7 +7682,7 @@
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr"/>
@@ -7771,7 +7771,7 @@
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr"/>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr"/>
@@ -7949,7 +7949,7 @@
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr"/>
@@ -8038,7 +8038,7 @@
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr"/>
@@ -8127,7 +8127,7 @@
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr"/>
@@ -8216,7 +8216,7 @@
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr"/>
@@ -8305,7 +8305,7 @@
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G86" s="3" t="inlineStr"/>
@@ -8394,7 +8394,7 @@
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr"/>
@@ -8483,7 +8483,7 @@
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr"/>
@@ -8572,7 +8572,7 @@
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr"/>
@@ -8661,7 +8661,7 @@
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr"/>
@@ -8750,7 +8750,7 @@
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G91" s="3" t="inlineStr"/>
@@ -8839,7 +8839,7 @@
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G92" s="3" t="inlineStr"/>
@@ -8928,7 +8928,7 @@
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G93" s="3" t="inlineStr"/>
@@ -9017,7 +9017,7 @@
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G94" s="3" t="inlineStr"/>
@@ -9106,7 +9106,7 @@
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G95" s="3" t="inlineStr"/>
@@ -9195,7 +9195,7 @@
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G96" s="3" t="inlineStr"/>
@@ -9284,7 +9284,7 @@
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G97" s="3" t="inlineStr"/>
@@ -9373,7 +9373,7 @@
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G98" s="3" t="inlineStr"/>
@@ -9462,7 +9462,7 @@
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G99" s="3" t="inlineStr"/>
@@ -9551,7 +9551,7 @@
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G100" s="3" t="inlineStr"/>
@@ -9640,7 +9640,7 @@
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G101" s="3" t="inlineStr"/>
@@ -9729,7 +9729,7 @@
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr"/>
@@ -9818,7 +9818,7 @@
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G103" s="3" t="inlineStr"/>
@@ -9907,7 +9907,7 @@
       </c>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G104" s="3" t="inlineStr"/>
@@ -9996,7 +9996,7 @@
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G105" s="3" t="inlineStr"/>
@@ -10085,7 +10085,7 @@
       </c>
       <c r="F106" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G106" s="3" t="inlineStr"/>
@@ -10174,7 +10174,7 @@
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G107" s="3" t="inlineStr"/>
@@ -10263,7 +10263,7 @@
       </c>
       <c r="F108" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G108" s="3" t="inlineStr"/>
@@ -10352,7 +10352,7 @@
       </c>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G109" s="3" t="inlineStr"/>
@@ -10441,7 +10441,7 @@
       </c>
       <c r="F110" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G110" s="3" t="inlineStr"/>
@@ -10530,7 +10530,7 @@
       </c>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G111" s="3" t="inlineStr"/>
@@ -10619,7 +10619,7 @@
       </c>
       <c r="F112" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G112" s="3" t="inlineStr"/>
@@ -10708,7 +10708,7 @@
       </c>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G113" s="3" t="inlineStr"/>
@@ -10797,7 +10797,7 @@
       </c>
       <c r="F114" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G114" s="3" t="inlineStr"/>
@@ -10886,7 +10886,7 @@
       </c>
       <c r="F115" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G115" s="3" t="inlineStr"/>
@@ -10975,7 +10975,7 @@
       </c>
       <c r="F116" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G116" s="3" t="inlineStr"/>
@@ -11064,7 +11064,7 @@
       </c>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G117" s="3" t="inlineStr"/>
@@ -11153,7 +11153,7 @@
       </c>
       <c r="F118" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G118" s="3" t="inlineStr"/>
@@ -11242,7 +11242,7 @@
       </c>
       <c r="F119" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G119" s="3" t="inlineStr"/>
@@ -11331,7 +11331,7 @@
       </c>
       <c r="F120" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G120" s="3" t="inlineStr"/>
@@ -11420,7 +11420,7 @@
       </c>
       <c r="F121" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G121" s="3" t="inlineStr"/>
@@ -11509,7 +11509,7 @@
       </c>
       <c r="F122" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G122" s="3" t="inlineStr"/>
@@ -11598,7 +11598,7 @@
       </c>
       <c r="F123" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G123" s="3" t="inlineStr"/>
@@ -11687,7 +11687,7 @@
       </c>
       <c r="F124" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G124" s="3" t="inlineStr"/>
@@ -11776,7 +11776,7 @@
       </c>
       <c r="F125" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G125" s="3" t="inlineStr"/>
@@ -11865,7 +11865,7 @@
       </c>
       <c r="F126" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G126" s="3" t="inlineStr"/>
@@ -11954,7 +11954,7 @@
       </c>
       <c r="F127" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G127" s="3" t="inlineStr"/>
@@ -12043,7 +12043,7 @@
       </c>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G128" s="3" t="inlineStr"/>
@@ -12132,7 +12132,7 @@
       </c>
       <c r="F129" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G129" s="3" t="inlineStr"/>
@@ -12221,7 +12221,7 @@
       </c>
       <c r="F130" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G130" s="3" t="inlineStr"/>
@@ -12310,7 +12310,7 @@
       </c>
       <c r="F131" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G131" s="3" t="inlineStr"/>
@@ -12399,7 +12399,7 @@
       </c>
       <c r="F132" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G132" s="3" t="inlineStr"/>
@@ -12488,7 +12488,7 @@
       </c>
       <c r="F133" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G133" s="3" t="inlineStr"/>
@@ -12577,7 +12577,7 @@
       </c>
       <c r="F134" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G134" s="3" t="inlineStr"/>
@@ -12666,7 +12666,7 @@
       </c>
       <c r="F135" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G135" s="3" t="inlineStr"/>
@@ -12755,7 +12755,7 @@
       </c>
       <c r="F136" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G136" s="3" t="inlineStr"/>
@@ -12844,7 +12844,7 @@
       </c>
       <c r="F137" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G137" s="3" t="inlineStr"/>
@@ -12933,7 +12933,7 @@
       </c>
       <c r="F138" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G138" s="3" t="inlineStr"/>
@@ -13022,7 +13022,7 @@
       </c>
       <c r="F139" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G139" s="3" t="inlineStr"/>
@@ -13111,7 +13111,7 @@
       </c>
       <c r="F140" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G140" s="3" t="inlineStr"/>
@@ -13200,7 +13200,7 @@
       </c>
       <c r="F141" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G141" s="3" t="inlineStr"/>
@@ -13289,7 +13289,7 @@
       </c>
       <c r="F142" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G142" s="3" t="inlineStr"/>
@@ -13378,7 +13378,7 @@
       </c>
       <c r="F143" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G143" s="3" t="inlineStr"/>
@@ -13467,7 +13467,7 @@
       </c>
       <c r="F144" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G144" s="3" t="inlineStr"/>
@@ -13556,7 +13556,7 @@
       </c>
       <c r="F145" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G145" s="3" t="inlineStr"/>
@@ -13645,7 +13645,7 @@
       </c>
       <c r="F146" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G146" s="3" t="inlineStr"/>
@@ -13734,7 +13734,7 @@
       </c>
       <c r="F147" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G147" s="3" t="inlineStr"/>
@@ -13823,7 +13823,7 @@
       </c>
       <c r="F148" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G148" s="3" t="inlineStr"/>
@@ -13912,7 +13912,7 @@
       </c>
       <c r="F149" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G149" s="3" t="inlineStr"/>
@@ -14001,7 +14001,7 @@
       </c>
       <c r="F150" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G150" s="3" t="inlineStr"/>
@@ -14090,7 +14090,7 @@
       </c>
       <c r="F151" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G151" s="3" t="inlineStr"/>
@@ -14179,7 +14179,7 @@
       </c>
       <c r="F152" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G152" s="3" t="inlineStr"/>
@@ -14268,7 +14268,7 @@
       </c>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G153" s="3" t="inlineStr"/>
@@ -14357,7 +14357,7 @@
       </c>
       <c r="F154" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G154" s="3" t="inlineStr"/>
@@ -14446,7 +14446,7 @@
       </c>
       <c r="F155" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G155" s="3" t="inlineStr"/>
@@ -14535,7 +14535,7 @@
       </c>
       <c r="F156" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G156" s="3" t="inlineStr"/>
@@ -14624,7 +14624,7 @@
       </c>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G157" s="3" t="inlineStr"/>
@@ -14713,7 +14713,7 @@
       </c>
       <c r="F158" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G158" s="3" t="inlineStr"/>
@@ -14802,7 +14802,7 @@
       </c>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G159" s="3" t="inlineStr"/>
@@ -14891,7 +14891,7 @@
       </c>
       <c r="F160" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G160" s="3" t="inlineStr"/>
@@ -14980,7 +14980,7 @@
       </c>
       <c r="F161" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G161" s="3" t="inlineStr"/>
@@ -15069,7 +15069,7 @@
       </c>
       <c r="F162" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G162" s="3" t="inlineStr"/>
@@ -15158,7 +15158,7 @@
       </c>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G163" s="3" t="inlineStr"/>
@@ -15247,7 +15247,7 @@
       </c>
       <c r="F164" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G164" s="3" t="inlineStr"/>
@@ -15336,7 +15336,7 @@
       </c>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G165" s="3" t="inlineStr"/>
@@ -15425,7 +15425,7 @@
       </c>
       <c r="F166" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G166" s="3" t="inlineStr">
@@ -15518,7 +15518,7 @@
       </c>
       <c r="F167" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G167" s="3" t="inlineStr">
@@ -15611,7 +15611,7 @@
       </c>
       <c r="F168" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G168" s="3" t="inlineStr">
@@ -15704,7 +15704,7 @@
       </c>
       <c r="F169" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G169" s="3" t="inlineStr">
@@ -15797,7 +15797,7 @@
       </c>
       <c r="F170" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G170" s="3" t="inlineStr"/>
@@ -15886,7 +15886,7 @@
       </c>
       <c r="F171" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G171" s="3" t="inlineStr">
@@ -15979,7 +15979,7 @@
       </c>
       <c r="F172" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G172" s="3" t="inlineStr">
@@ -16072,7 +16072,7 @@
       </c>
       <c r="F173" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G173" s="3" t="inlineStr">
@@ -16165,7 +16165,7 @@
       </c>
       <c r="F174" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G174" s="3" t="inlineStr"/>
@@ -16254,7 +16254,7 @@
       </c>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G175" s="3" t="inlineStr"/>
@@ -16343,7 +16343,7 @@
       </c>
       <c r="F176" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G176" s="3" t="inlineStr"/>
@@ -16432,7 +16432,7 @@
       </c>
       <c r="F177" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G177" s="3" t="inlineStr"/>
@@ -16521,7 +16521,7 @@
       </c>
       <c r="F178" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G178" s="3" t="inlineStr">
@@ -16614,7 +16614,7 @@
       </c>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G179" s="3" t="inlineStr">
@@ -16707,7 +16707,7 @@
       </c>
       <c r="F180" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G180" s="3" t="inlineStr">
@@ -16800,7 +16800,7 @@
       </c>
       <c r="F181" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G181" s="3" t="inlineStr">
@@ -16893,7 +16893,7 @@
       </c>
       <c r="F182" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G182" s="3" t="inlineStr">
@@ -16986,7 +16986,7 @@
       </c>
       <c r="F183" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G183" s="3" t="inlineStr">
@@ -17079,7 +17079,7 @@
       </c>
       <c r="F184" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G184" s="3" t="inlineStr"/>
@@ -17168,7 +17168,7 @@
       </c>
       <c r="F185" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G185" s="3" t="inlineStr"/>
@@ -17257,7 +17257,7 @@
       </c>
       <c r="F186" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G186" s="3" t="inlineStr"/>
@@ -17346,7 +17346,7 @@
       </c>
       <c r="F187" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G187" s="3" t="inlineStr"/>
@@ -17435,7 +17435,7 @@
       </c>
       <c r="F188" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G188" s="3" t="inlineStr"/>
@@ -17524,7 +17524,7 @@
       </c>
       <c r="F189" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G189" s="3" t="inlineStr"/>
@@ -17613,7 +17613,7 @@
       </c>
       <c r="F190" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G190" s="3" t="inlineStr"/>
@@ -17702,7 +17702,7 @@
       </c>
       <c r="F191" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G191" s="3" t="inlineStr"/>
@@ -17791,7 +17791,7 @@
       </c>
       <c r="F192" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G192" s="3" t="inlineStr"/>

</xml_diff>